<commit_message>
Update data files - Bot run at 2026-02-14 05:33:50 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,68 +425,106 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>user_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>username</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>level</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>last_message_date</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>last_response</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>response_status</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>level_3_ai_response</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>subscription_checked</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>level_4_reminder_sent</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>decision</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>first_added_date</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>6365338077</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>xman1221</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-02-14T05:33:17.871136+00:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Added during extraction</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-02-14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-02-15 01:57:05 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -528,6 +528,44 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>7059362073</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Arush23456</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>unreachable</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="b">
+        <v>0</v>
+      </c>
+      <c r="I3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Added during extraction</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-02-15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-02-16 01:53:32 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -575,6 +575,44 @@
       <c r="L3" t="inlineStr">
         <is>
           <t>2026-02-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>5890041990</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Yadavkunal97</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>unreachable</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="b">
+        <v>0</v>
+      </c>
+      <c r="I4" t="b">
+        <v>0</v>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Added during extraction</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-02-16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-02-16 11:38:51 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -500,11 +500,11 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-02-15T10:53:38.508692+00:00</t>
+          <t>2026-02-16T11:38:42.053720+00:00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -526,7 +526,7 @@
         <v>0</v>
       </c>
       <c r="I2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-02-17 01:52:03 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -613,6 +613,44 @@
       <c r="L4" t="inlineStr">
         <is>
           <t>2026-02-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1432292618</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>user_1432292618</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>unreachable</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="b">
+        <v>0</v>
+      </c>
+      <c r="I5" t="b">
+        <v>0</v>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Added during extraction</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-02-18 01:56:02 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -651,6 +651,44 @@
       <c r="L5" t="inlineStr">
         <is>
           <t>2026-02-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5789748925</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Meoneeei</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>unreachable</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="b">
+        <v>0</v>
+      </c>
+      <c r="I6" t="b">
+        <v>0</v>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Added during extraction</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-02-20 01:50:54 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -727,6 +727,40 @@
       <c r="L7" t="inlineStr">
         <is>
           <t>2026-02-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1549816407</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>probably_pratyush</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="b">
+        <v>0</v>
+      </c>
+      <c r="I8" t="b">
+        <v>0</v>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Added during extraction</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-02-22 01:54:14 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -798,6 +798,40 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>6660497489</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Helloooo_18</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="b">
+        <v>0</v>
+      </c>
+      <c r="I10" t="b">
+        <v>0</v>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Added during extraction</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-02-22</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-02-26 01:51:56 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -934,6 +934,40 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>8620686461</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>alex_ggmongg</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="b">
+        <v>0</v>
+      </c>
+      <c r="I14" t="b">
+        <v>0</v>
+      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Added during extraction</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-02-28 01:31:23 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1002,6 +1002,40 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>7289843412</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>user_7289843412</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="b">
+        <v>0</v>
+      </c>
+      <c r="I16" t="b">
+        <v>0</v>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Added during extraction</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-03-02 01:52:18 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1070,6 +1070,40 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>2020153141</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>islayadmins</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="b">
+        <v>0</v>
+      </c>
+      <c r="I18" t="b">
+        <v>0</v>
+      </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Added during extraction</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-03-03 01:54:29 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1104,6 +1104,40 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>6234770619</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>user_6234770619</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="b">
+        <v>0</v>
+      </c>
+      <c r="I19" t="b">
+        <v>0</v>
+      </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Added during extraction</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-03-05 01:51:59 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1172,6 +1172,40 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>7915742060</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>user_7915742060</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="b">
+        <v>0</v>
+      </c>
+      <c r="I21" t="b">
+        <v>0</v>
+      </c>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Added during extraction</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-03-07 01:44:26 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1240,6 +1240,40 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>6477064253</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>shubhi037</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="b">
+        <v>0</v>
+      </c>
+      <c r="I23" t="b">
+        <v>0</v>
+      </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Added during extraction</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-03-08 01:52:13 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1274,6 +1274,40 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>6352388699</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>user_6352388699</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="b">
+        <v>0</v>
+      </c>
+      <c r="I24" t="b">
+        <v>0</v>
+      </c>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Added during extraction</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-03-09 01:53:24 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1308,6 +1308,40 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>924160594</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>user_924160594</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="b">
+        <v>0</v>
+      </c>
+      <c r="I25" t="b">
+        <v>0</v>
+      </c>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Added during extraction</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-03-10 08:46:56 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1342,6 +1342,40 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>7339503030</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Phonix457</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="b">
+        <v>0</v>
+      </c>
+      <c r="I26" t="b">
+        <v>0</v>
+      </c>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Added during extraction</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-03-12 01:49:35 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1410,6 +1410,40 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>5350007972</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Manu9752</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="b">
+        <v>0</v>
+      </c>
+      <c r="I28" t="b">
+        <v>0</v>
+      </c>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Added during extraction</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-03-13 01:50:11 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1444,6 +1444,40 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>5089780638</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>sanvi1803</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="b">
+        <v>0</v>
+      </c>
+      <c r="I29" t="b">
+        <v>0</v>
+      </c>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Added during extraction</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-03-15 02:04:17 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1512,6 +1512,40 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>8017866965</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>user_8017866965</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="b">
+        <v>0</v>
+      </c>
+      <c r="I31" t="b">
+        <v>0</v>
+      </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Added during extraction</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-03-17 05:43:29 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -550,9 +550,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>-1</v>
-      </c>
-      <c r="D3" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-03-17T05:41:31.208872+00:00</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
@@ -588,9 +592,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>-1</v>
-      </c>
-      <c r="D4" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-03-17T05:41:49.860251+00:00</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
@@ -664,9 +672,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>-1</v>
-      </c>
-      <c r="D6" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-03-17T05:42:24.936199+00:00</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
@@ -702,9 +714,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>-1</v>
-      </c>
-      <c r="D7" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-03-17T05:42:45.588433+00:00</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-03-17 19:56:51 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -818,9 +818,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>-1</v>
-      </c>
-      <c r="D9" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-03-17T19:54:58.128139+00:00</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
@@ -856,9 +860,13 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>-1</v>
-      </c>
-      <c r="D10" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-03-17T19:55:18.929898+00:00</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-03-17 21:36:54 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -1058,9 +1058,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>-1</v>
-      </c>
-      <c r="D15" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026-03-17T21:36:12.137502+00:00</t>
+        </is>
+      </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-03-18 01:57:28 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1702,6 +1702,40 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>5551259677</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>user_5551259677</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="b">
+        <v>0</v>
+      </c>
+      <c r="I34" t="b">
+        <v>0</v>
+      </c>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Added during extraction</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-03-18 08:45:11 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -1020,9 +1020,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>-1</v>
-      </c>
-      <c r="D14" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026-03-18T08:44:01.344999+00:00</t>
+        </is>
+      </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-03-18 09:52:44 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -1146,9 +1146,13 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>-1</v>
-      </c>
-      <c r="D17" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2026-03-18T09:51:48.935758+00:00</t>
+        </is>
+      </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-03-18 11:44:48 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -1222,9 +1222,13 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>-1</v>
-      </c>
-      <c r="D19" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2026-03-18T11:43:54.385862+00:00</t>
+        </is>
+      </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-03-18 13:05:16 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -1260,9 +1260,13 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>-1</v>
-      </c>
-      <c r="D20" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2026-03-18T13:04:20.480717+00:00</t>
+        </is>
+      </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-03-18 14:48:14 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -1302,7 +1302,11 @@
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>unreachable</t>
+        </is>
+      </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-03-19 01:58:07 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1768,6 +1768,40 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>7908942533</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>user_7908942533</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="b">
+        <v>0</v>
+      </c>
+      <c r="I35" t="b">
+        <v>0</v>
+      </c>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Added during extraction</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update data files - Bot run at 2026-04-13 13:21:44 UTC
</commit_message>
<xml_diff>
--- a/dm_promotion_service/data/users_engagement.xlsx
+++ b/dm_promotion_service/data/users_engagement.xlsx
@@ -826,11 +826,11 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-04-12T12:57:25.584701+00:00</t>
+          <t>2026-04-13T13:21:27.854224+00:00</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -852,7 +852,7 @@
         <v>0</v>
       </c>
       <c r="I9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">

</xml_diff>